<commit_message>
anova reemplazado por no parametricos
</commit_message>
<xml_diff>
--- a/output/tables/table_1_anual_2.0.xlsx
+++ b/output/tables/table_1_anual_2.0.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0.316</t>
+          <t>0.365</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0.316</t>
+          <t>0.365</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.316</t>
+          <t>0.365</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.041 *</t>
+          <t>0.012 *</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0.041 *</t>
+          <t>0.012 *</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.041 *</t>
+          <t>0.012 *</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0.188</t>
+          <t>0.441</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.188</t>
+          <t>0.441</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.188</t>
+          <t>0.441</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0.002 *</t>
+          <t>0.336</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0.002 *</t>
+          <t>0.336</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.002 *</t>
+          <t>0.336</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.123</t>
+          <t>0.169</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.123</t>
+          <t>0.169</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.123</t>
+          <t>0.169</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0.005 *</t>
+          <t>0.035 *</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.005 *</t>
+          <t>0.035 *</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.005 *</t>
+          <t>0.035 *</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.607</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.607</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.607</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.127</t>
+          <t>0.741</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0.127</t>
+          <t>0.741</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.127</t>
+          <t>0.741</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0.006 *</t>
+          <t>0.273</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0.006 *</t>
+          <t>0.273</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0.006 *</t>
+          <t>0.273</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0.014 *</t>
+          <t>0.006 *</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0.014 *</t>
+          <t>0.006 *</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.014 *</t>
+          <t>0.006 *</t>
         </is>
       </c>
     </row>

</xml_diff>